<commit_message>
Reduce features to 37 per mentor feedback
</commit_message>
<xml_diff>
--- a/lstm_features.xlsx
+++ b/lstm_features.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D70"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -776,7 +776,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>resp_fio2_(%)</t>
+          <t>resp_fio2</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Respiratory charting: fio2 (%)</t>
+          <t>Respiratory charting: fio2</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>resp_fio2</t>
+          <t>resp_peep</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -808,7 +808,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Respiratory charting: fio2</t>
+          <t>Respiratory charting: peep</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>resp_peep</t>
+          <t>age</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Respiratory charting: peep</t>
+          <t>Patient age (years, capped at 90)</t>
         </is>
       </c>
     </row>
@@ -842,17 +842,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>resp_peep/cpap</t>
+          <t>diag_Diabetes</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Continuous</t>
+          <t>Binary</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Respiratory charting: peep/cpap</t>
+          <t>Binary flag: 1 if patient diagnosed with Diabetes</t>
         </is>
       </c>
     </row>
@@ -864,17 +864,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>resp_ps_above_peep</t>
+          <t>diag_Hypertension</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Continuous</t>
+          <t>Binary</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Respiratory charting: ps above peep</t>
+          <t>Binary flag: 1 if patient diagnosed with Hypertension</t>
         </is>
       </c>
     </row>
@@ -886,17 +886,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>resp_set_fraction_of_inspired_oxygen_(fio2)</t>
+          <t>diag_Heart_Disease</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Continuous</t>
+          <t>Binary</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Respiratory charting: set fraction of inspired oxygen (fio2)</t>
+          <t>Binary flag: 1 if patient diagnosed with Heart Disease</t>
         </is>
       </c>
     </row>
@@ -908,17 +908,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>resp_unable_to_obtain_peepi_and_vtrap</t>
+          <t>diag_Kidney_Disease</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Continuous</t>
+          <t>Binary</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Respiratory charting: unable to obtain peepi and vtrap</t>
+          <t>Binary flag: 1 if patient diagnosed with Kidney Disease</t>
         </is>
       </c>
     </row>
@@ -930,17 +930,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>age</t>
+          <t>diag_Sepsis</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Continuous</t>
+          <t>Binary</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Patient age (years, capped at 90)</t>
+          <t>Binary flag: 1 if patient diagnosed with Sepsis</t>
         </is>
       </c>
     </row>
@@ -952,17 +952,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>admissionheight</t>
+          <t>diag_Pneumonia</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Continuous</t>
+          <t>Binary</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Height at admission (cm)</t>
+          <t>Binary flag: 1 if patient diagnosed with Pneumonia</t>
         </is>
       </c>
     </row>
@@ -974,17 +974,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>admissionweight</t>
+          <t>diag_COPD</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Continuous</t>
+          <t>Binary</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Weight at admission (kg)</t>
+          <t>Binary flag: 1 if patient diagnosed with COPD</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>diag_Diabetes</t>
+          <t>diag_Liver_Disease</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Binary flag: 1 if patient diagnosed with Diabetes</t>
+          <t>Binary flag: 1 if patient diagnosed with Liver Disease</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>diag_Hypertension</t>
+          <t>med_Antibiotics</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Binary flag: 1 if patient diagnosed with Hypertension</t>
+          <t>Binary flag: 1 if patient received Antibiotics</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>diag_Heart_Disease</t>
+          <t>med_Vasopressors</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Binary flag: 1 if patient diagnosed with Heart Disease</t>
+          <t>Binary flag: 1 if patient received Vasopressors</t>
         </is>
       </c>
     </row>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>diag_Kidney_Disease</t>
+          <t>med_Sedatives</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Binary flag: 1 if patient diagnosed with Kidney Disease</t>
+          <t>Binary flag: 1 if patient received Sedatives</t>
         </is>
       </c>
     </row>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>diag_Sepsis</t>
+          <t>med_Insulin</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Binary flag: 1 if patient diagnosed with Sepsis</t>
+          <t>Binary flag: 1 if patient received Insulin</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>diag_Pneumonia</t>
+          <t>med_Anticoagulants</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Binary flag: 1 if patient diagnosed with Pneumonia</t>
+          <t>Binary flag: 1 if patient received Anticoagulants</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>diag_COPD</t>
+          <t>med_Steroids</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Binary flag: 1 if patient diagnosed with COPD</t>
+          <t>Binary flag: 1 if patient received Steroids</t>
         </is>
       </c>
     </row>
@@ -1150,17 +1150,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>diag_Liver_Disease</t>
+          <t>bmi</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Binary</t>
+          <t>Continuous</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Binary flag: 1 if patient diagnosed with Liver Disease</t>
+          <t>Body Mass Index = weight / (height/100)^2</t>
         </is>
       </c>
     </row>
@@ -1172,17 +1172,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>med_Antibiotics</t>
+          <t>pulse_pressure</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Binary</t>
+          <t>Continuous</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Binary flag: 1 if patient received Antibiotics</t>
+          <t>Systolic - Diastolic blood pressure</t>
         </is>
       </c>
     </row>
@@ -1194,17 +1194,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>med_Vasopressors</t>
+          <t>map_calculated</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Binary</t>
+          <t>Continuous</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Binary flag: 1 if patient received Vasopressors</t>
+          <t>Calculated Mean Arterial Pressure</t>
         </is>
       </c>
     </row>
@@ -1216,17 +1216,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>med_Sedatives</t>
+          <t>shock_index</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Binary</t>
+          <t>Continuous</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Binary flag: 1 if patient received Sedatives</t>
+          <t>Heart Rate / Systolic Blood Pressure</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>med_Insulin</t>
+          <t>gender_Male</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1248,711 +1248,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Binary flag: 1 if patient received Insulin</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>med_Anticoagulants</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Binary flag: 1 if patient received Anticoagulants</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>med_Steroids</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Binary flag: 1 if patient received Steroids</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>40</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>bmi</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Body Mass Index = weight / (height/100)^2</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>41</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>pulse_pressure</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Systolic - Diastolic blood pressure</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>map_calculated</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Calculated Mean Arterial Pressure</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>43</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>shock_index</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>Heart Rate / Systolic Blood Pressure</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>heartrate_rolling_mean</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>6-hour rolling mean of heartrate</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>heartrate_rolling_std</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>6-hour rolling standard deviation of heartrate</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>46</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>heartrate_rate_of_change</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Hour-over-hour change in heartrate</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>47</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>systemicsystolic_rolling_mean</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>6-hour rolling mean of systemicsystolic</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>48</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>systemicsystolic_rolling_std</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>6-hour rolling standard deviation of systemicsystolic</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>49</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>systemicsystolic_rate_of_change</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Hour-over-hour change in systemicsystolic</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>systemicdiastolic_rolling_mean</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>6-hour rolling mean of systemicdiastolic</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>51</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>systemicdiastolic_rolling_std</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>6-hour rolling standard deviation of systemicdiastolic</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>52</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>systemicdiastolic_rate_of_change</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Hour-over-hour change in systemicdiastolic</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>53</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>systemicmean_rolling_mean</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>6-hour rolling mean of systemicmean</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>54</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>systemicmean_rolling_std</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>6-hour rolling standard deviation of systemicmean</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>systemicmean_rate_of_change</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Hour-over-hour change in systemicmean</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>56</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>respiration_rolling_mean</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>6-hour rolling mean of respiration</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>57</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>respiration_rolling_std</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>6-hour rolling standard deviation of respiration</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>58</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>respiration_rate_of_change</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Hour-over-hour change in respiration</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>59</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>temperature_rolling_mean</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>6-hour rolling mean of temperature</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>temperature_rolling_std</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>6-hour rolling standard deviation of temperature</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>61</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>temperature_rate_of_change</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Continuous</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Hour-over-hour change in temperature</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>62</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>gender_Female</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>One-hot encoded gender: Female</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>gender_Male</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
           <t>One-hot encoded gender: Male</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>64</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>ethnicity_African American</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>One-hot encoded ethnicity: African American</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>65</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>ethnicity_Asian</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>One-hot encoded ethnicity: Asian</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>66</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>ethnicity_Caucasian</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>One-hot encoded ethnicity: Caucasian</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>67</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>ethnicity_Hispanic</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>One-hot encoded ethnicity: Hispanic</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>68</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>ethnicity_Native American</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>One-hot encoded ethnicity: Native American</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>69</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>ethnicity_Other/Unknown</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Binary</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>One-hot encoded ethnicity: Other/Unknown</t>
         </is>
       </c>
     </row>

</xml_diff>